<commit_message>
Monthly labor update - Jan 2026
</commit_message>
<xml_diff>
--- a/Data/Labor and Employment/Labor and Employment.xlsx
+++ b/Data/Labor and Employment/Labor and Employment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Labor and Employment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7446202-AF14-4406-BD4E-53F12C57526D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEECC5B0-10CB-40BA-A997-9F462A4129CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3023" uniqueCount="839">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3091" uniqueCount="855">
   <si>
     <t>LFS Round</t>
   </si>
@@ -2555,6 +2555,54 @@
   </si>
   <si>
     <t>https://psa.gov.ph/content/number-unemployed-persons-december-2025-increased-226-million-filipinos-aged-15-years-and</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/number-unemployed-persons-january-2026-increased-296-million-filipinos-aged-15-years-and</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>2026 Jan</t>
+  </si>
+  <si>
+    <t>2026 Feb</t>
+  </si>
+  <si>
+    <t>2026 Mar</t>
+  </si>
+  <si>
+    <t>2026 Apr</t>
+  </si>
+  <si>
+    <t>2026 May</t>
+  </si>
+  <si>
+    <t>2026 Jun</t>
+  </si>
+  <si>
+    <t>2026 Jul</t>
+  </si>
+  <si>
+    <t>2026 Aug</t>
+  </si>
+  <si>
+    <t>2026 Sep</t>
+  </si>
+  <si>
+    <t>2026 Oct</t>
+  </si>
+  <si>
+    <t>2026 Nov</t>
+  </si>
+  <si>
+    <t>2026 Dec</t>
+  </si>
+  <si>
+    <t>2026 Annual</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/2024-annual-provincial-labor-market-statistics-preliminary-results</t>
   </si>
 </sst>
 </file>
@@ -3023,7 +3071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P299"/>
+  <dimension ref="A1:P312"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="1" customWidth="1"/>
@@ -15507,7 +15555,7 @@
         <v>2157.422</v>
       </c>
       <c r="N274" s="2">
-        <f t="shared" ref="N274:N299" si="34">J274-K274</f>
+        <f t="shared" ref="N274:N300" si="34">J274-K274</f>
         <v>30572.822</v>
       </c>
       <c r="O274" s="2">
@@ -16136,6 +16184,9 @@
       <c r="O286" s="2">
         <v>5818.1239999999998</v>
       </c>
+      <c r="P286" t="s">
+        <v>854</v>
+      </c>
     </row>
     <row r="287" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
@@ -16150,40 +16201,37 @@
       <c r="D287" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E287" s="1" t="s">
-        <v>425</v>
-      </c>
       <c r="F287" s="3">
         <f t="shared" ref="F287:F288" si="49">K287/J287</f>
-        <v>0.63860962824397194</v>
+        <v>0.63860613190398863</v>
       </c>
       <c r="G287" s="3">
         <f t="shared" ref="G287:G288" si="50">L287/K287</f>
-        <v>0.95726078411505899</v>
+        <v>0.95725210956042472</v>
       </c>
       <c r="H287" s="3">
         <f t="shared" ref="H287:H288" si="51">M287/K287</f>
-        <v>4.2739215884941006E-2</v>
+        <v>4.2747890439575394E-2</v>
       </c>
       <c r="I287" s="3">
         <f t="shared" ref="I287:I288" si="52">O287/L287</f>
         <v>0.13342662775918007</v>
       </c>
       <c r="J287" s="2">
-        <v>79315.19</v>
+        <v>79316.342999999993</v>
       </c>
       <c r="K287" s="2">
-        <v>50651.444000000003</v>
+        <v>50651.902999999998</v>
       </c>
       <c r="L287" s="2">
         <v>48486.641000000003</v>
       </c>
       <c r="M287" s="2">
-        <v>2164.8029999999999</v>
+        <v>2165.2620000000002</v>
       </c>
       <c r="N287" s="2">
         <f t="shared" si="34"/>
-        <v>28663.745999999999</v>
+        <v>28664.439999999995</v>
       </c>
       <c r="O287" s="2">
         <v>6469.4089999999997</v>
@@ -16847,6 +16895,232 @@
       </c>
       <c r="O299" s="2">
         <v>5823.357</v>
+      </c>
+    </row>
+    <row r="300" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A300" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C300" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D300" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E300" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="F300" s="3">
+        <f t="shared" ref="F300" si="81">K300/J300</f>
+        <v>0.62304594527350909</v>
+      </c>
+      <c r="G300" s="3">
+        <f t="shared" ref="G300" si="82">L300/K300</f>
+        <v>0.94193643540031868</v>
+      </c>
+      <c r="H300" s="3">
+        <f t="shared" ref="H300" si="83">M300/K300</f>
+        <v>5.8063564599681317E-2</v>
+      </c>
+      <c r="I300" s="3">
+        <f t="shared" ref="I300" si="84">O300/L300</f>
+        <v>0.13244881397687053</v>
+      </c>
+      <c r="J300" s="2">
+        <v>81683.548999999999</v>
+      </c>
+      <c r="K300" s="2">
+        <v>50892.603999999999</v>
+      </c>
+      <c r="L300" s="2">
+        <v>47937.597999999998</v>
+      </c>
+      <c r="M300" s="2">
+        <v>2955.0059999999999</v>
+      </c>
+      <c r="N300" s="2">
+        <f t="shared" si="34"/>
+        <v>30790.945</v>
+      </c>
+      <c r="O300" s="2">
+        <v>6349.2780000000002</v>
+      </c>
+      <c r="P300" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="301" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A301" s="1" t="s">
+        <v>842</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C301" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="D301" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="302" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A302" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C302" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D302" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E302" s="36"/>
+    </row>
+    <row r="303" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A303" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C303" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D303" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E303" s="37"/>
+    </row>
+    <row r="304" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A304" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C304" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D304" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A305" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C305" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="D305" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A306" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C306" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D306" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E306" s="48"/>
+    </row>
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A307" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C307" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="D307" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A308" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C308" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="D308" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A309" s="1" t="s">
+        <v>850</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C309" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D309" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A310" s="1" t="s">
+        <v>851</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C310" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="D310" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A311" s="1" t="s">
+        <v>852</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C311" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D311" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A312" s="1" t="s">
+        <v>853</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="C312" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D312" s="1" t="s">
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -48125,7 +48399,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D191"/>
+  <dimension ref="A1:D204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" style="1" customWidth="1"/>
@@ -49908,6 +50182,74 @@
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>779</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="B192" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193" s="1" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194" s="1" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195" s="1" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196" s="1" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197" s="1" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198" s="1" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199" s="1" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200" s="1" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201" s="1" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202" s="1" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203" s="1" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
+        <v>853</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monthly labor update - Feb 2026
</commit_message>
<xml_diff>
--- a/Data/Labor and Employment/Labor and Employment.xlsx
+++ b/Data/Labor and Employment/Labor and Employment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Labor and Employment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEECC5B0-10CB-40BA-A997-9F462A4129CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBD6C23C-45E3-4851-948F-FE91F0022072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9345" yWindow="3240" windowWidth="12705" windowHeight="11940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compiled" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3091" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3094" uniqueCount="857">
   <si>
     <t>LFS Round</t>
   </si>
@@ -2603,6 +2603,12 @@
   </si>
   <si>
     <t>https://psa.gov.ph/content/2024-annual-provincial-labor-market-statistics-preliminary-results</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/2025-annual-provincial-labor-market-statistics-preliminary-results</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/unemployment-rate-declined-51-percent-labor-market-conditions-improved-february-2026</t>
   </si>
 </sst>
 </file>
@@ -15555,7 +15561,7 @@
         <v>2157.422</v>
       </c>
       <c r="N274" s="2">
-        <f t="shared" ref="N274:N300" si="34">J274-K274</f>
+        <f t="shared" ref="N274:N301" si="34">J274-K274</f>
         <v>30572.822</v>
       </c>
       <c r="O274" s="2">
@@ -16253,40 +16259,37 @@
       <c r="D288" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E288" s="1" t="s">
-        <v>425</v>
-      </c>
       <c r="F288" s="3">
         <f t="shared" si="49"/>
-        <v>0.64473209315915503</v>
+        <v>0.64472798115191687</v>
       </c>
       <c r="G288" s="3">
         <f t="shared" si="50"/>
-        <v>0.96208863606203909</v>
+        <v>0.96208534683068936</v>
       </c>
       <c r="H288" s="3">
         <f t="shared" si="51"/>
-        <v>3.7911363937960858E-2</v>
+        <v>3.7914672741739958E-2</v>
       </c>
       <c r="I288" s="3">
         <f t="shared" si="52"/>
-        <v>0.1008763827044134</v>
+        <v>0.10087542842932454</v>
       </c>
       <c r="J288" s="2">
-        <v>79244.729000000007</v>
+        <v>79246.255000000005</v>
       </c>
       <c r="K288" s="2">
-        <v>51091.62</v>
+        <v>51092.277999999998</v>
       </c>
       <c r="L288" s="2">
-        <v>49154.667000000001</v>
+        <v>49155.131999999998</v>
       </c>
       <c r="M288" s="2">
-        <v>1936.953</v>
+        <v>1937.1469999999999</v>
       </c>
       <c r="N288" s="2">
         <f t="shared" si="34"/>
-        <v>28153.109000000004</v>
+        <v>28153.977000000006</v>
       </c>
       <c r="O288" s="2">
         <v>4958.5450000000001</v>
@@ -16896,6 +16899,9 @@
       <c r="O299" s="2">
         <v>5823.357</v>
       </c>
+      <c r="P299" t="s">
+        <v>855</v>
+      </c>
     </row>
     <row r="300" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
@@ -16964,6 +16970,44 @@
       </c>
       <c r="D301" s="1" t="s">
         <v>417</v>
+      </c>
+      <c r="F301" s="3">
+        <f t="shared" ref="F301" si="85">K301/J301</f>
+        <v>0.63814578496183227</v>
+      </c>
+      <c r="G301" s="3">
+        <f t="shared" ref="G301" si="86">L301/K301</f>
+        <v>0.94891847087590342</v>
+      </c>
+      <c r="H301" s="3">
+        <f t="shared" ref="H301" si="87">M301/K301</f>
+        <v>5.1081529124096595E-2</v>
+      </c>
+      <c r="I301" s="3">
+        <f t="shared" ref="I301" si="88">O301/L301</f>
+        <v>0.1181406960296031</v>
+      </c>
+      <c r="J301" s="2">
+        <v>81621.751999999993</v>
+      </c>
+      <c r="K301" s="2">
+        <v>52086.576999999997</v>
+      </c>
+      <c r="L301" s="2">
+        <v>49425.915000000001</v>
+      </c>
+      <c r="M301" s="2">
+        <v>2660.6619999999998</v>
+      </c>
+      <c r="N301" s="2">
+        <f t="shared" si="34"/>
+        <v>29535.174999999996</v>
+      </c>
+      <c r="O301" s="2">
+        <v>5839.2120000000004</v>
+      </c>
+      <c r="P301" t="s">
+        <v>856</v>
       </c>
     </row>
     <row r="302" spans="1:16" x14ac:dyDescent="0.25">
@@ -50183,6 +50227,9 @@
       <c r="A191" s="1" t="s">
         <v>779</v>
       </c>
+      <c r="B191" t="s">
+        <v>855</v>
+      </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
@@ -50192,62 +50239,65 @@
         <v>839</v>
       </c>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>842</v>
       </c>
-    </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B193" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>843</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>844</v>
       </c>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>846</v>
       </c>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>847</v>
       </c>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>849</v>
       </c>
     </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>851</v>
       </c>
     </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>853</v>
       </c>

</xml_diff>

<commit_message>
Monthly labor update - Mar 2026
</commit_message>
<xml_diff>
--- a/Data/Labor and Employment/Labor and Employment.xlsx
+++ b/Data/Labor and Employment/Labor and Employment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Labor and Employment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBD6C23C-45E3-4851-948F-FE91F0022072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C369442-94CB-470E-A441-C6008CEBCAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9345" yWindow="3240" windowWidth="12705" windowHeight="11940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compiled" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3094" uniqueCount="857">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3095" uniqueCount="858">
   <si>
     <t>LFS Round</t>
   </si>
@@ -2609,6 +2609,9 @@
   </si>
   <si>
     <t>https://psa.gov.ph/content/unemployment-rate-declined-51-percent-labor-market-conditions-improved-february-2026</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/unemployment-rate-eased-50-percent-march-2026</t>
   </si>
 </sst>
 </file>
@@ -15561,7 +15564,7 @@
         <v>2157.422</v>
       </c>
       <c r="N274" s="2">
-        <f t="shared" ref="N274:N301" si="34">J274-K274</f>
+        <f t="shared" ref="N274:N302" si="34">J274-K274</f>
         <v>30572.822</v>
       </c>
       <c r="O274" s="2">
@@ -16311,43 +16314,41 @@
       <c r="D289" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E289" s="36" t="s">
-        <v>425</v>
-      </c>
+      <c r="E289" s="36"/>
       <c r="F289" s="3">
         <f t="shared" ref="F289" si="53">K289/J289</f>
-        <v>0.62855197137035979</v>
+        <v>0.62852465692284698</v>
       </c>
       <c r="G289" s="3">
         <f t="shared" ref="G289" si="54">L289/K289</f>
-        <v>0.96133642592656232</v>
+        <v>0.96132601706253951</v>
       </c>
       <c r="H289" s="3">
         <f t="shared" ref="H289" si="55">M289/K289</f>
-        <v>3.8663574073437589E-2</v>
+        <v>3.8673982937460612E-2</v>
       </c>
       <c r="I289" s="3">
         <f t="shared" ref="I289" si="56">O289/L289</f>
-        <v>0.13404737188395227</v>
+        <v>0.1340917865241773</v>
       </c>
       <c r="J289" s="2">
-        <v>79478.47</v>
+        <v>79478.551000000007</v>
       </c>
       <c r="K289" s="2">
-        <v>49956.349000000002</v>
+        <v>49954.228999999999</v>
       </c>
       <c r="L289" s="2">
-        <v>48024.858</v>
+        <v>48022.3</v>
       </c>
       <c r="M289" s="2">
-        <v>1931.491</v>
+        <v>1931.9290000000001</v>
       </c>
       <c r="N289" s="2">
         <f t="shared" si="34"/>
-        <v>29522.120999999999</v>
+        <v>29524.322000000007</v>
       </c>
       <c r="O289" s="2">
-        <v>6437.6059999999998</v>
+        <v>6439.3959999999997</v>
       </c>
       <c r="P289" t="s">
         <v>783</v>
@@ -17024,6 +17025,44 @@
         <v>417</v>
       </c>
       <c r="E302" s="36"/>
+      <c r="F302" s="3">
+        <f t="shared" ref="F302" si="89">K302/J302</f>
+        <v>0.63323252936195007</v>
+      </c>
+      <c r="G302" s="3">
+        <f t="shared" ref="G302" si="90">L302/K302</f>
+        <v>0.95010655661650911</v>
+      </c>
+      <c r="H302" s="3">
+        <f t="shared" ref="H302" si="91">M302/K302</f>
+        <v>4.9893443383490894E-2</v>
+      </c>
+      <c r="I302" s="3">
+        <f t="shared" ref="I302" si="92">O302/L302</f>
+        <v>0.12291139509308913</v>
+      </c>
+      <c r="J302" s="2">
+        <v>81558.956000000006</v>
+      </c>
+      <c r="K302" s="2">
+        <v>51645.784</v>
+      </c>
+      <c r="L302" s="2">
+        <v>49068.998</v>
+      </c>
+      <c r="M302" s="2">
+        <v>2576.7860000000001</v>
+      </c>
+      <c r="N302" s="2">
+        <f t="shared" si="34"/>
+        <v>29913.172000000006</v>
+      </c>
+      <c r="O302" s="2">
+        <v>6031.1390000000001</v>
+      </c>
+      <c r="P302" t="s">
+        <v>857</v>
+      </c>
     </row>
     <row r="303" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
@@ -17039,6 +17078,7 @@
         <v>417</v>
       </c>
       <c r="E303" s="37"/>
+      <c r="O303" s="2"/>
     </row>
     <row r="304" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
@@ -17053,8 +17093,9 @@
       <c r="D304" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O304" s="2"/>
+    </row>
+    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
         <v>846</v>
       </c>
@@ -17067,8 +17108,9 @@
       <c r="D305" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O305" s="2"/>
+    </row>
+    <row r="306" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
         <v>847</v>
       </c>
@@ -17082,8 +17124,9 @@
         <v>417</v>
       </c>
       <c r="E306" s="48"/>
-    </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O306" s="2"/>
+    </row>
+    <row r="307" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
         <v>848</v>
       </c>
@@ -17096,8 +17139,9 @@
       <c r="D307" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O307" s="2"/>
+    </row>
+    <row r="308" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
         <v>849</v>
       </c>
@@ -17110,8 +17154,9 @@
       <c r="D308" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O308" s="2"/>
+    </row>
+    <row r="309" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
         <v>850</v>
       </c>
@@ -17124,8 +17169,9 @@
       <c r="D309" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O309" s="2"/>
+    </row>
+    <row r="310" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
         <v>851</v>
       </c>
@@ -17138,8 +17184,9 @@
       <c r="D310" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O310" s="2"/>
+    </row>
+    <row r="311" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
         <v>852</v>
       </c>
@@ -17152,8 +17199,9 @@
       <c r="D311" s="1" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="O311" s="2"/>
+    </row>
+    <row r="312" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
         <v>853</v>
       </c>
@@ -17166,6 +17214,7 @@
       <c r="D312" s="1" t="s">
         <v>417</v>
       </c>
+      <c r="O312" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -50251,6 +50300,9 @@
       <c r="A194" s="1" t="s">
         <v>843</v>
       </c>
+      <c r="B194" t="s">
+        <v>857</v>
+      </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">

</xml_diff>

<commit_message>
Monthly labor update - April 2026
</commit_message>
<xml_diff>
--- a/Data/Labor and Employment/Labor and Employment.xlsx
+++ b/Data/Labor and Employment/Labor and Employment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Labor and Employment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C369442-94CB-470E-A441-C6008CEBCAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABE9B2A5-578D-4E23-8577-C68B2B749966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2700" yWindow="2340" windowWidth="15780" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compiled" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3095" uniqueCount="858">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3103" uniqueCount="863">
   <si>
     <t>LFS Round</t>
   </si>
@@ -2612,6 +2612,21 @@
   </si>
   <si>
     <t>https://psa.gov.ph/content/unemployment-rate-eased-50-percent-march-2026</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/number-employed-persons-april-2026-increased-4889-million-filipinos-aged-15-years-and-over</t>
+  </si>
+  <si>
+    <t>2026Apr</t>
+  </si>
+  <si>
+    <t>2026Mar</t>
+  </si>
+  <si>
+    <t>2026Feb</t>
+  </si>
+  <si>
+    <t>2026Jan</t>
   </si>
 </sst>
 </file>
@@ -2624,11 +2639,18 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2783,11 +2805,11 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2812,44 +2834,47 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -15564,7 +15589,7 @@
         <v>2157.422</v>
       </c>
       <c r="N274" s="2">
-        <f t="shared" ref="N274:N302" si="34">J274-K274</f>
+        <f t="shared" ref="N274:N303" si="34">J274-K274</f>
         <v>30572.822</v>
       </c>
       <c r="O274" s="2">
@@ -16367,9 +16392,7 @@
       <c r="D290" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E290" s="37" t="s">
-        <v>425</v>
-      </c>
+      <c r="E290" s="37"/>
       <c r="F290" s="3">
         <f t="shared" ref="F290" si="57">K290/J290</f>
         <v>0.63744363097856882</v>
@@ -16972,6 +16995,9 @@
       <c r="D301" s="1" t="s">
         <v>417</v>
       </c>
+      <c r="E301" s="1" t="s">
+        <v>425</v>
+      </c>
       <c r="F301" s="3">
         <f t="shared" ref="F301" si="85">K301/J301</f>
         <v>0.63814578496183227</v>
@@ -17024,7 +17050,9 @@
       <c r="D302" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E302" s="36"/>
+      <c r="E302" s="51" t="s">
+        <v>425</v>
+      </c>
       <c r="F302" s="3">
         <f t="shared" ref="F302" si="89">K302/J302</f>
         <v>0.63323252936195007</v>
@@ -17077,8 +17105,47 @@
       <c r="D303" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E303" s="37"/>
-      <c r="O303" s="2"/>
+      <c r="E303" s="51" t="s">
+        <v>425</v>
+      </c>
+      <c r="F303" s="3">
+        <f t="shared" ref="F303" si="93">K303/J303</f>
+        <v>0.62680754809337047</v>
+      </c>
+      <c r="G303" s="3">
+        <f t="shared" ref="G303" si="94">L303/K303</f>
+        <v>0.95294387941059833</v>
+      </c>
+      <c r="H303" s="3">
+        <f t="shared" ref="H303" si="95">M303/K303</f>
+        <v>4.7056120589401763E-2</v>
+      </c>
+      <c r="I303" s="3">
+        <f t="shared" ref="I303" si="96">O303/L303</f>
+        <v>0.15157325103830141</v>
+      </c>
+      <c r="J303" s="2">
+        <v>81849.066999999995</v>
+      </c>
+      <c r="K303" s="2">
+        <v>51303.612999999998</v>
+      </c>
+      <c r="L303" s="2">
+        <v>48889.464</v>
+      </c>
+      <c r="M303" s="2">
+        <v>2414.1489999999999</v>
+      </c>
+      <c r="N303" s="2">
+        <f t="shared" si="34"/>
+        <v>30545.453999999998</v>
+      </c>
+      <c r="O303" s="2">
+        <v>7410.335</v>
+      </c>
+      <c r="P303" t="s">
+        <v>858</v>
+      </c>
     </row>
     <row r="304" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
@@ -20473,7 +20540,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="12" type="noConversion"/>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -20481,16 +20548,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0B3FDD3-8CAB-4986-8439-B73CD0CD9872}">
-  <dimension ref="A1:CE54"/>
+  <dimension ref="A1:CI54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.5703125" style="24" customWidth="1"/>
     <col min="2" max="71" width="10.7109375" style="24" customWidth="1"/>
-    <col min="72" max="83" width="10.7109375" style="26" customWidth="1"/>
-    <col min="84" max="16384" width="9.140625" style="24"/>
+    <col min="72" max="87" width="10.7109375" style="26" customWidth="1"/>
+    <col min="88" max="16384" width="9.140625" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
         <v>685</v>
       </c>
@@ -20701,7 +20768,7 @@
       <c r="BR1" s="35" t="s">
         <v>764</v>
       </c>
-      <c r="BS1" s="51" t="s">
+      <c r="BS1" s="53" t="s">
         <v>766</v>
       </c>
       <c r="BT1" s="26" t="s">
@@ -20713,7 +20780,7 @@
       <c r="BV1" s="26" t="s">
         <v>824</v>
       </c>
-      <c r="BW1" s="26" t="s">
+      <c r="BW1" s="52" t="s">
         <v>825</v>
       </c>
       <c r="BX1" s="26" t="s">
@@ -20740,8 +20807,20 @@
       <c r="CE1" s="50" t="s">
         <v>833</v>
       </c>
-    </row>
-    <row r="2" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF1" s="54" t="s">
+        <v>862</v>
+      </c>
+      <c r="CG1" s="54" t="s">
+        <v>861</v>
+      </c>
+      <c r="CH1" s="54" t="s">
+        <v>860</v>
+      </c>
+      <c r="CI1" s="54" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="2" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
         <v>694</v>
       </c>
@@ -20927,10 +21006,10 @@
         <v>48486.641000000003</v>
       </c>
       <c r="BU2" s="34">
-        <v>49154.667000000001</v>
+        <v>49155.131999999998</v>
       </c>
       <c r="BV2" s="34">
-        <v>48024.858</v>
+        <v>48022.3</v>
       </c>
       <c r="BW2" s="34">
         <v>48671.648000000001</v>
@@ -20959,8 +21038,20 @@
       <c r="CE2" s="26">
         <v>49427.023999999998</v>
       </c>
-    </row>
-    <row r="3" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF2" s="34">
+        <v>47937.597999999998</v>
+      </c>
+      <c r="CG2" s="34">
+        <v>49425.915000000001</v>
+      </c>
+      <c r="CH2" s="34">
+        <v>49068.998</v>
+      </c>
+      <c r="CI2" s="34">
+        <v>48889.464</v>
+      </c>
+    </row>
+    <row r="3" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A3" s="28" t="s">
         <v>691</v>
       </c>
@@ -21031,7 +21122,7 @@
       <c r="BR3" s="26"/>
       <c r="BS3" s="26"/>
     </row>
-    <row r="4" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>693</v>
       </c>
@@ -21214,16 +21305,16 @@
         <v>9439.6910000000007</v>
       </c>
       <c r="BT4" s="26">
-        <v>8936.34</v>
+        <v>8934.3719999999994</v>
       </c>
       <c r="BU4" s="26">
-        <v>8415.9940000000006</v>
+        <v>8418.3580000000002</v>
       </c>
       <c r="BV4" s="26">
-        <v>8470.4310000000005</v>
+        <v>8471.7170000000006</v>
       </c>
       <c r="BW4" s="26">
-        <v>8612.8130000000001</v>
+        <v>8610.2610000000004</v>
       </c>
       <c r="BX4" s="26">
         <v>9431.5139999999992</v>
@@ -21249,8 +21340,20 @@
       <c r="CE4" s="26">
         <v>9273.0519999999997</v>
       </c>
-    </row>
-    <row r="5" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF4" s="26">
+        <v>7515.3950000000004</v>
+      </c>
+      <c r="CG4" s="26">
+        <v>7895.0129999999999</v>
+      </c>
+      <c r="CH4" s="26">
+        <v>8381.5079999999998</v>
+      </c>
+      <c r="CI4" s="26">
+        <v>8218.6059999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>692</v>
       </c>
@@ -21433,7 +21536,7 @@
         <v>1223.2280000000001</v>
       </c>
       <c r="BT5" s="26">
-        <v>1308.03</v>
+        <v>1307.856</v>
       </c>
       <c r="BU5" s="26">
         <v>1455.258</v>
@@ -21468,8 +21571,20 @@
       <c r="CE5" s="26">
         <v>965.60599999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF5" s="26">
+        <v>1168.0509999999999</v>
+      </c>
+      <c r="CG5" s="26">
+        <v>1400.816</v>
+      </c>
+      <c r="CH5" s="26">
+        <v>980.77700000000004</v>
+      </c>
+      <c r="CI5" s="26">
+        <v>1253.923</v>
+      </c>
+    </row>
+    <row r="6" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
         <v>685</v>
       </c>
@@ -21538,7 +21653,7 @@
       <c r="BR6" s="26"/>
       <c r="BS6" s="26"/>
     </row>
-    <row r="7" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>690</v>
       </c>
@@ -21721,7 +21836,7 @@
         <v>291.67200000000003</v>
       </c>
       <c r="BT7" s="26">
-        <v>221.58500000000001</v>
+        <v>220.392</v>
       </c>
       <c r="BU7" s="26">
         <v>231.15100000000001</v>
@@ -21730,7 +21845,7 @@
         <v>177.78700000000001</v>
       </c>
       <c r="BW7" s="26">
-        <v>188.47800000000001</v>
+        <v>187.976</v>
       </c>
       <c r="BX7" s="26">
         <v>167.53</v>
@@ -21756,8 +21871,20 @@
       <c r="CE7" s="26">
         <v>210.66499999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF7" s="26">
+        <v>257.41500000000002</v>
+      </c>
+      <c r="CG7" s="26">
+        <v>247.14099999999999</v>
+      </c>
+      <c r="CH7" s="26">
+        <v>324.60000000000002</v>
+      </c>
+      <c r="CI7" s="26">
+        <v>346.44799999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
         <v>689</v>
       </c>
@@ -21940,16 +22067,16 @@
         <v>3402.808</v>
       </c>
       <c r="BT8" s="26">
-        <v>3360.5790000000002</v>
+        <v>3367.7240000000002</v>
       </c>
       <c r="BU8" s="26">
-        <v>3585.5050000000001</v>
+        <v>3585.096</v>
       </c>
       <c r="BV8" s="26">
-        <v>3700.2350000000001</v>
+        <v>3695.4119999999998</v>
       </c>
       <c r="BW8" s="26">
-        <v>3328.8119999999999</v>
+        <v>3327.5920000000001</v>
       </c>
       <c r="BX8" s="26">
         <v>3513.08</v>
@@ -21975,8 +22102,20 @@
       <c r="CE8" s="26">
         <v>3147.6930000000002</v>
       </c>
-    </row>
-    <row r="9" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF8" s="26">
+        <v>3693.7040000000002</v>
+      </c>
+      <c r="CG8" s="26">
+        <v>3763.319</v>
+      </c>
+      <c r="CH8" s="26">
+        <v>3546.7910000000002</v>
+      </c>
+      <c r="CI8" s="26">
+        <v>3587.0659999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
         <v>688</v>
       </c>
@@ -22162,13 +22301,13 @@
         <v>88.766999999999996</v>
       </c>
       <c r="BU9" s="26">
-        <v>94.613</v>
+        <v>94.67</v>
       </c>
       <c r="BV9" s="26">
         <v>84.483000000000004</v>
       </c>
       <c r="BW9" s="26">
-        <v>112.11499999999999</v>
+        <v>110.288</v>
       </c>
       <c r="BX9" s="26">
         <v>96.335999999999999</v>
@@ -22194,8 +22333,20 @@
       <c r="CE9" s="26">
         <v>115.184</v>
       </c>
-    </row>
-    <row r="10" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF9" s="26">
+        <v>107.005</v>
+      </c>
+      <c r="CG9" s="26">
+        <v>107.886</v>
+      </c>
+      <c r="CH9" s="26">
+        <v>100.622</v>
+      </c>
+      <c r="CI9" s="26">
+        <v>110.767</v>
+      </c>
+    </row>
+    <row r="10" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
         <v>687</v>
       </c>
@@ -22378,7 +22529,7 @@
         <v>55.939</v>
       </c>
       <c r="BT10" s="26">
-        <v>90.847999999999999</v>
+        <v>90.442999999999998</v>
       </c>
       <c r="BU10" s="26">
         <v>49.323</v>
@@ -22387,7 +22538,7 @@
         <v>67.367000000000004</v>
       </c>
       <c r="BW10" s="26">
-        <v>75.254000000000005</v>
+        <v>78.067999999999998</v>
       </c>
       <c r="BX10" s="26">
         <v>58.371000000000002</v>
@@ -22413,8 +22564,20 @@
       <c r="CE10" s="26">
         <v>71.676000000000002</v>
       </c>
-    </row>
-    <row r="11" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF10" s="26">
+        <v>102.398</v>
+      </c>
+      <c r="CG10" s="26">
+        <v>54.878999999999998</v>
+      </c>
+      <c r="CH10" s="26">
+        <v>84.019000000000005</v>
+      </c>
+      <c r="CI10" s="26">
+        <v>94.965000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
         <v>686</v>
       </c>
@@ -22600,13 +22763,13 @@
         <v>4596.8190000000004</v>
       </c>
       <c r="BU11" s="26">
-        <v>5031.027</v>
+        <v>5034.17</v>
       </c>
       <c r="BV11" s="26">
         <v>4558.4160000000002</v>
       </c>
       <c r="BW11" s="26">
-        <v>4810.8779999999997</v>
+        <v>4810.817</v>
       </c>
       <c r="BX11" s="26">
         <v>4785.1679999999997</v>
@@ -22632,8 +22795,20 @@
       <c r="CE11" s="26">
         <v>4796.9049999999997</v>
       </c>
-    </row>
-    <row r="12" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF11" s="26">
+        <v>4597.78</v>
+      </c>
+      <c r="CG11" s="26">
+        <v>4550.3280000000004</v>
+      </c>
+      <c r="CH11" s="26">
+        <v>4733.893</v>
+      </c>
+      <c r="CI11" s="26">
+        <v>4808.732</v>
+      </c>
+    </row>
+    <row r="12" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A12" s="28" t="s">
         <v>669</v>
       </c>
@@ -22702,7 +22877,7 @@
       <c r="BR12" s="26"/>
       <c r="BS12" s="26"/>
     </row>
-    <row r="13" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
         <v>683</v>
       </c>
@@ -22885,16 +23060,16 @@
         <v>10197.041999999999</v>
       </c>
       <c r="BT13" s="26">
-        <v>9991.3279999999995</v>
+        <v>9969.3510000000006</v>
       </c>
       <c r="BU13" s="26">
-        <v>10611.763999999999</v>
+        <v>10622.892</v>
       </c>
       <c r="BV13" s="26">
-        <v>10172.986000000001</v>
+        <v>9929.4509999999991</v>
       </c>
       <c r="BW13" s="26">
-        <v>10130.905000000001</v>
+        <v>10105.784</v>
       </c>
       <c r="BX13" s="26">
         <v>9940.4140000000007</v>
@@ -22920,8 +23095,20 @@
       <c r="CE13" s="26">
         <v>10128.037</v>
       </c>
-    </row>
-    <row r="14" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF13" s="26">
+        <v>9240.1880000000001</v>
+      </c>
+      <c r="CG13" s="26">
+        <v>9898.366</v>
+      </c>
+      <c r="CH13" s="26">
+        <v>9911.7520000000004</v>
+      </c>
+      <c r="CI13" s="26">
+        <v>9656.1389999999992</v>
+      </c>
+    </row>
+    <row r="14" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
         <v>682</v>
       </c>
@@ -23104,16 +23291,16 @@
         <v>4037.2950000000001</v>
       </c>
       <c r="BT14" s="26">
-        <v>3856.989</v>
+        <v>3857.31</v>
       </c>
       <c r="BU14" s="26">
-        <v>3680.9879999999998</v>
+        <v>3682.2550000000001</v>
       </c>
       <c r="BV14" s="26">
-        <v>3544.52</v>
+        <v>3545.6819999999998</v>
       </c>
       <c r="BW14" s="26">
-        <v>3768.9630000000002</v>
+        <v>3767.777</v>
       </c>
       <c r="BX14" s="26">
         <v>3746.1660000000002</v>
@@ -23139,8 +23326,20 @@
       <c r="CE14" s="26">
         <v>3778.9</v>
       </c>
-    </row>
-    <row r="15" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF14" s="26">
+        <v>4016.8910000000001</v>
+      </c>
+      <c r="CG14" s="26">
+        <v>4168.45</v>
+      </c>
+      <c r="CH14" s="26">
+        <v>4053.125</v>
+      </c>
+      <c r="CI14" s="26">
+        <v>3956.7249999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
         <v>681</v>
       </c>
@@ -23323,16 +23522,16 @@
         <v>2659.1289999999999</v>
       </c>
       <c r="BT15" s="26">
-        <v>2698.9050000000002</v>
+        <v>2715</v>
       </c>
       <c r="BU15" s="26">
-        <v>2815.482</v>
+        <v>2803.4749999999999</v>
       </c>
       <c r="BV15" s="26">
-        <v>2913.1869999999999</v>
+        <v>3166.7829999999999</v>
       </c>
       <c r="BW15" s="26">
-        <v>2567.8820000000001</v>
+        <v>2593.4250000000002</v>
       </c>
       <c r="BX15" s="26">
         <v>3347.152</v>
@@ -23358,8 +23557,20 @@
       <c r="CE15" s="26">
         <v>2939.3980000000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF15" s="26">
+        <v>2799.2539999999999</v>
+      </c>
+      <c r="CG15" s="26">
+        <v>3160.0189999999998</v>
+      </c>
+      <c r="CH15" s="26">
+        <v>3150.8020000000001</v>
+      </c>
+      <c r="CI15" s="26">
+        <v>3103.8670000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
         <v>680</v>
       </c>
@@ -23542,16 +23753,16 @@
         <v>487.00700000000001</v>
       </c>
       <c r="BT16" s="26">
-        <v>502.625</v>
+        <v>502.34500000000003</v>
       </c>
       <c r="BU16" s="26">
-        <v>413.47500000000002</v>
+        <v>416.47300000000001</v>
       </c>
       <c r="BV16" s="26">
-        <v>513.9</v>
+        <v>513.25300000000004</v>
       </c>
       <c r="BW16" s="26">
-        <v>454.27</v>
+        <v>452.30500000000001</v>
       </c>
       <c r="BX16" s="26">
         <v>500.88</v>
@@ -23577,8 +23788,20 @@
       <c r="CE16" s="26">
         <v>479.32</v>
       </c>
-    </row>
-    <row r="17" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF16" s="26">
+        <v>534.44899999999996</v>
+      </c>
+      <c r="CG16" s="26">
+        <v>469.30099999999999</v>
+      </c>
+      <c r="CH16" s="26">
+        <v>565.06399999999996</v>
+      </c>
+      <c r="CI16" s="26">
+        <v>490.93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
         <v>679</v>
       </c>
@@ -23761,16 +23984,16 @@
         <v>762.55499999999995</v>
       </c>
       <c r="BT17" s="26">
-        <v>742.65499999999997</v>
+        <v>742.78700000000003</v>
       </c>
       <c r="BU17" s="26">
-        <v>674.68499999999995</v>
+        <v>673.19600000000003</v>
       </c>
       <c r="BV17" s="26">
-        <v>687.39800000000002</v>
+        <v>686.87900000000002</v>
       </c>
       <c r="BW17" s="26">
-        <v>656.87800000000004</v>
+        <v>658.38199999999995</v>
       </c>
       <c r="BX17" s="26">
         <v>636.30899999999997</v>
@@ -23796,8 +24019,20 @@
       <c r="CE17" s="26">
         <v>677.22</v>
       </c>
-    </row>
-    <row r="18" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF17" s="26">
+        <v>728.08600000000001</v>
+      </c>
+      <c r="CG17" s="26">
+        <v>896.75699999999995</v>
+      </c>
+      <c r="CH17" s="26">
+        <v>780.95500000000004</v>
+      </c>
+      <c r="CI17" s="26">
+        <v>744.93799999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
         <v>678</v>
       </c>
@@ -23980,13 +24215,13 @@
         <v>334.19099999999997</v>
       </c>
       <c r="BT18" s="26">
-        <v>282.58199999999999</v>
+        <v>280.822</v>
       </c>
       <c r="BU18" s="26">
-        <v>211.39699999999999</v>
+        <v>212.18700000000001</v>
       </c>
       <c r="BV18" s="26">
-        <v>268.63499999999999</v>
+        <v>262.30099999999999</v>
       </c>
       <c r="BW18" s="26">
         <v>272.22199999999998</v>
@@ -24015,8 +24250,20 @@
       <c r="CE18" s="26">
         <v>300.92500000000001</v>
       </c>
-    </row>
-    <row r="19" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF18" s="26">
+        <v>274.21100000000001</v>
+      </c>
+      <c r="CG18" s="26">
+        <v>272.73700000000002</v>
+      </c>
+      <c r="CH18" s="26">
+        <v>307.05900000000003</v>
+      </c>
+      <c r="CI18" s="26">
+        <v>282.81099999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>677</v>
       </c>
@@ -24199,16 +24446,16 @@
         <v>438.92700000000002</v>
       </c>
       <c r="BT19" s="26">
-        <v>427.60500000000002</v>
+        <v>426.68900000000002</v>
       </c>
       <c r="BU19" s="26">
-        <v>337.34399999999999</v>
+        <v>337.40199999999999</v>
       </c>
       <c r="BV19" s="26">
         <v>271.33499999999998</v>
       </c>
       <c r="BW19" s="26">
-        <v>392.25</v>
+        <v>391.28399999999999</v>
       </c>
       <c r="BX19" s="26">
         <v>465.33199999999999</v>
@@ -24234,8 +24481,20 @@
       <c r="CE19" s="26">
         <v>441.21600000000001</v>
       </c>
-    </row>
-    <row r="20" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF19" s="26">
+        <v>486.67200000000003</v>
+      </c>
+      <c r="CG19" s="26">
+        <v>389.46699999999998</v>
+      </c>
+      <c r="CH19" s="26">
+        <v>480.75900000000001</v>
+      </c>
+      <c r="CI19" s="26">
+        <v>378.964</v>
+      </c>
+    </row>
+    <row r="20" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
         <v>676</v>
       </c>
@@ -24418,16 +24677,16 @@
         <v>2534.0810000000001</v>
       </c>
       <c r="BT20" s="26">
-        <v>2686.248</v>
+        <v>2691.9009999999998</v>
       </c>
       <c r="BU20" s="26">
-        <v>2378.7370000000001</v>
+        <v>2453.951</v>
       </c>
       <c r="BV20" s="26">
-        <v>2560.5210000000002</v>
+        <v>2560.7049999999999</v>
       </c>
       <c r="BW20" s="26">
-        <v>3005.9679999999998</v>
+        <v>3008.3760000000002</v>
       </c>
       <c r="BX20" s="26">
         <v>2791.047</v>
@@ -24453,8 +24712,20 @@
       <c r="CE20" s="26">
         <v>2918.683</v>
       </c>
-    </row>
-    <row r="21" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF20" s="26">
+        <v>3094.864</v>
+      </c>
+      <c r="CG20" s="26">
+        <v>3025.8049999999998</v>
+      </c>
+      <c r="CH20" s="26">
+        <v>3018.433</v>
+      </c>
+      <c r="CI20" s="26">
+        <v>2958.6370000000002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
         <v>675</v>
       </c>
@@ -24637,16 +24908,16 @@
         <v>3132.174</v>
       </c>
       <c r="BT21" s="26">
-        <v>2820.9369999999999</v>
+        <v>2819.0740000000001</v>
       </c>
       <c r="BU21" s="26">
-        <v>3011.819</v>
+        <v>2949.6309999999999</v>
       </c>
       <c r="BV21" s="26">
-        <v>2853.5650000000001</v>
+        <v>2855.279</v>
       </c>
       <c r="BW21" s="26">
-        <v>3063.433</v>
+        <v>3065.34</v>
       </c>
       <c r="BX21" s="26">
         <v>3049.3209999999999</v>
@@ -24672,8 +24943,20 @@
       <c r="CE21" s="26">
         <v>3215.5920000000001</v>
       </c>
-    </row>
-    <row r="22" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF21" s="26">
+        <v>3160.5990000000002</v>
+      </c>
+      <c r="CG21" s="26">
+        <v>2824.107</v>
+      </c>
+      <c r="CH21" s="26">
+        <v>2717.8029999999999</v>
+      </c>
+      <c r="CI21" s="26">
+        <v>3015.7750000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
         <v>674</v>
       </c>
@@ -24856,16 +25139,16 @@
         <v>1585.222</v>
       </c>
       <c r="BT22" s="26">
-        <v>1585.1379999999999</v>
+        <v>1591.529</v>
       </c>
       <c r="BU22" s="26">
-        <v>1668.931</v>
+        <v>1650.162</v>
       </c>
       <c r="BV22" s="26">
-        <v>1825.681</v>
+        <v>1823.97</v>
       </c>
       <c r="BW22" s="26">
-        <v>1632.9159999999999</v>
+        <v>1630.933</v>
       </c>
       <c r="BX22" s="26">
         <v>1783.15</v>
@@ -24891,8 +25174,20 @@
       <c r="CE22" s="26">
         <v>1826.231</v>
       </c>
-    </row>
-    <row r="23" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF22" s="26">
+        <v>1672.4290000000001</v>
+      </c>
+      <c r="CG22" s="26">
+        <v>1750.7249999999999</v>
+      </c>
+      <c r="CH22" s="26">
+        <v>1892.867</v>
+      </c>
+      <c r="CI22" s="26">
+        <v>1737.954</v>
+      </c>
+    </row>
+    <row r="23" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
         <v>673</v>
       </c>
@@ -25075,16 +25370,16 @@
         <v>848.83399999999995</v>
       </c>
       <c r="BT23" s="26">
-        <v>744.32100000000003</v>
+        <v>738.35199999999998</v>
       </c>
       <c r="BU23" s="26">
-        <v>739.54399999999998</v>
+        <v>764.09100000000001</v>
       </c>
       <c r="BV23" s="26">
-        <v>729.77099999999996</v>
+        <v>727.83799999999997</v>
       </c>
       <c r="BW23" s="26">
-        <v>779.73900000000003</v>
+        <v>783.79899999999998</v>
       </c>
       <c r="BX23" s="26">
         <v>723.24400000000003</v>
@@ -25110,8 +25405,20 @@
       <c r="CE23" s="26">
         <v>758.62</v>
       </c>
-    </row>
-    <row r="24" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF23" s="26">
+        <v>824.98199999999997</v>
+      </c>
+      <c r="CG23" s="26">
+        <v>978.47400000000005</v>
+      </c>
+      <c r="CH23" s="26">
+        <v>824.15200000000004</v>
+      </c>
+      <c r="CI23" s="26">
+        <v>758.59199999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
         <v>672</v>
       </c>
@@ -25294,16 +25601,16 @@
         <v>406.45100000000002</v>
       </c>
       <c r="BT24" s="26">
-        <v>442.35599999999999</v>
+        <v>441.14499999999998</v>
       </c>
       <c r="BU24" s="26">
-        <v>517.08199999999999</v>
+        <v>513.55700000000002</v>
       </c>
       <c r="BV24" s="26">
-        <v>514.57500000000005</v>
+        <v>514.23</v>
       </c>
       <c r="BW24" s="26">
-        <v>446.09800000000001</v>
+        <v>445.36599999999999</v>
       </c>
       <c r="BX24" s="26">
         <v>504.75099999999998</v>
@@ -25329,8 +25636,20 @@
       <c r="CE24" s="26">
         <v>450.40899999999999</v>
       </c>
-    </row>
-    <row r="25" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF24" s="26">
+        <v>482.51299999999998</v>
+      </c>
+      <c r="CG24" s="26">
+        <v>427.36799999999999</v>
+      </c>
+      <c r="CH24" s="26">
+        <v>367.56200000000001</v>
+      </c>
+      <c r="CI24" s="26">
+        <v>466.43299999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
         <v>671</v>
       </c>
@@ -25513,16 +25832,16 @@
         <v>2935.0390000000002</v>
       </c>
       <c r="BT25" s="26">
-        <v>3099.953</v>
+        <v>3101.9340000000002</v>
       </c>
       <c r="BU25" s="26">
-        <v>3230.55</v>
+        <v>3207.8330000000001</v>
       </c>
       <c r="BV25" s="26">
-        <v>2940.152</v>
+        <v>2939.4969999999998</v>
       </c>
       <c r="BW25" s="26">
-        <v>2962.739</v>
+        <v>2962.6170000000002</v>
       </c>
       <c r="BX25" s="26">
         <v>3225.5749999999998</v>
@@ -25548,8 +25867,20 @@
       <c r="CE25" s="26">
         <v>2931.6880000000001</v>
       </c>
-    </row>
-    <row r="26" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF25" s="26">
+        <v>3179.8470000000002</v>
+      </c>
+      <c r="CG25" s="26">
+        <v>3143.88</v>
+      </c>
+      <c r="CH25" s="26">
+        <v>2845.0410000000002</v>
+      </c>
+      <c r="CI25" s="26">
+        <v>2917.0720000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>670</v>
       </c>
@@ -25767,8 +26098,20 @@
       <c r="CE26" s="26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:83" x14ac:dyDescent="0.25">
+      <c r="CF26" s="26">
+        <v>0.86599999999999999</v>
+      </c>
+      <c r="CG26" s="26">
+        <v>1.0780000000000001</v>
+      </c>
+      <c r="CH26" s="26">
+        <v>1.415</v>
+      </c>
+      <c r="CI26" s="26">
+        <v>0.11899999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A27" s="28" t="s">
         <v>694</v>
       </c>
@@ -25875,7 +26218,7 @@
       <c r="BR27" s="26"/>
       <c r="BS27" s="26"/>
     </row>
-    <row r="28" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A28" s="28" t="s">
         <v>691</v>
       </c>
@@ -25954,7 +26297,7 @@
       <c r="BR28" s="26"/>
       <c r="BS28" s="26"/>
     </row>
-    <row r="29" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
         <v>693</v>
       </c>
@@ -26061,7 +26404,7 @@
       <c r="BR29" s="26"/>
       <c r="BS29" s="26"/>
     </row>
-    <row r="30" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
         <v>692</v>
       </c>
@@ -26168,7 +26511,7 @@
       <c r="BR30" s="26"/>
       <c r="BS30" s="26"/>
     </row>
-    <row r="31" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A31" s="28" t="s">
         <v>685</v>
       </c>
@@ -26246,7 +26589,7 @@
       <c r="BR31" s="26"/>
       <c r="BS31" s="26"/>
     </row>
-    <row r="32" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A32" s="25" t="s">
         <v>690</v>
       </c>
@@ -50308,6 +50651,9 @@
       <c r="A195" s="1" t="s">
         <v>844</v>
       </c>
+      <c r="B195" t="s">
+        <v>858</v>
+      </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">

</xml_diff>

<commit_message>
Monthly labor update - May 2026
</commit_message>
<xml_diff>
--- a/Data/Labor and Employment/Labor and Employment.xlsx
+++ b/Data/Labor and Employment/Labor and Employment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Labor and Employment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABE9B2A5-578D-4E23-8577-C68B2B749966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFA572A-9E60-4F04-8E65-778ECDE79733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="2340" windowWidth="15780" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compiled" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3103" uniqueCount="863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3105" uniqueCount="864">
   <si>
     <t>LFS Round</t>
   </si>
@@ -2627,6 +2627,9 @@
   </si>
   <si>
     <t>2026Jan</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/underemployment-rate-declined-122-percent-may-2026</t>
   </si>
 </sst>
 </file>
@@ -2639,11 +2642,18 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2805,11 +2815,11 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2834,47 +2844,48 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="10" fillId="6" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -15589,7 +15600,7 @@
         <v>2157.422</v>
       </c>
       <c r="N274" s="2">
-        <f t="shared" ref="N274:N303" si="34">J274-K274</f>
+        <f t="shared" ref="N274:N304" si="34">J274-K274</f>
         <v>30572.822</v>
       </c>
       <c r="O274" s="2">
@@ -16445,9 +16456,6 @@
       <c r="D291" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E291" s="1" t="s">
-        <v>425</v>
-      </c>
       <c r="F291" s="3">
         <f t="shared" ref="F291" si="61">K291/J291</f>
         <v>0.6584863836337842</v>
@@ -17160,7 +17168,47 @@
       <c r="D304" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="O304" s="2"/>
+      <c r="E304" s="55" t="s">
+        <v>425</v>
+      </c>
+      <c r="F304" s="3">
+        <f t="shared" ref="F304" si="97">K304/J304</f>
+        <v>0.63811943802781423</v>
+      </c>
+      <c r="G304" s="3">
+        <f t="shared" ref="G304" si="98">L304/K304</f>
+        <v>0.95207138197787045</v>
+      </c>
+      <c r="H304" s="3">
+        <f t="shared" ref="H304" si="99">M304/K304</f>
+        <v>4.7928618022129568E-2</v>
+      </c>
+      <c r="I304" s="3">
+        <f t="shared" ref="I304" si="100">O304/L304</f>
+        <v>0.12167668102712879</v>
+      </c>
+      <c r="J304" s="2">
+        <v>81686.178</v>
+      </c>
+      <c r="K304" s="2">
+        <v>52125.538</v>
+      </c>
+      <c r="L304" s="2">
+        <v>49627.233</v>
+      </c>
+      <c r="M304" s="2">
+        <v>2498.3049999999998</v>
+      </c>
+      <c r="N304" s="2">
+        <f t="shared" si="34"/>
+        <v>29560.639999999999</v>
+      </c>
+      <c r="O304" s="2">
+        <v>6038.4769999999999</v>
+      </c>
+      <c r="P304" t="s">
+        <v>863</v>
+      </c>
     </row>
     <row r="305" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
@@ -20540,7 +20588,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -50659,6 +50707,9 @@
       <c r="A196" s="1" t="s">
         <v>845</v>
       </c>
+      <c r="B196" t="s">
+        <v>863</v>
+      </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">

</xml_diff>

<commit_message>
Monthly labor update - June 2026
</commit_message>
<xml_diff>
--- a/Data/Labor and Employment/Labor and Employment.xlsx
+++ b/Data/Labor and Employment/Labor and Employment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Labor and Employment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFA572A-9E60-4F04-8E65-778ECDE79733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADFB279-7AA5-42A8-BFFD-989B765819B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compiled" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3105" uniqueCount="864">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3107" uniqueCount="865">
   <si>
     <t>LFS Round</t>
   </si>
@@ -2630,6 +2630,9 @@
   </si>
   <si>
     <t>https://psa.gov.ph/content/underemployment-rate-declined-122-percent-may-2026</t>
+  </si>
+  <si>
+    <t>https://psa.gov.ph/content/number-employed-persons-increased-5066-million-labor-force-participation-rose-june-2026</t>
   </si>
 </sst>
 </file>
@@ -15600,7 +15603,7 @@
         <v>2157.422</v>
       </c>
       <c r="N274" s="2">
-        <f t="shared" ref="N274:N304" si="34">J274-K274</f>
+        <f t="shared" ref="N274:N305" si="34">J274-K274</f>
         <v>30572.822</v>
       </c>
       <c r="O274" s="2">
@@ -16508,9 +16511,6 @@
       <c r="D292" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E292" s="1" t="s">
-        <v>425</v>
-      </c>
       <c r="F292" s="3">
         <f t="shared" ref="F292:F295" si="65">K292/J292</f>
         <v>0.65710331091544816</v>
@@ -17210,7 +17210,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
         <v>846</v>
       </c>
@@ -17223,9 +17223,49 @@
       <c r="D305" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="O305" s="2"/>
-    </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E305" s="55" t="s">
+        <v>425</v>
+      </c>
+      <c r="F305" s="3">
+        <f t="shared" ref="F305" si="101">K305/J305</f>
+        <v>0.65102425546943377</v>
+      </c>
+      <c r="G305" s="3">
+        <f t="shared" ref="G305" si="102">L305/K305</f>
+        <v>0.95140136141094411</v>
+      </c>
+      <c r="H305" s="3">
+        <f t="shared" ref="H305" si="103">M305/K305</f>
+        <v>4.859863858905588E-2</v>
+      </c>
+      <c r="I305" s="3">
+        <f t="shared" ref="I305" si="104">O305/L305</f>
+        <v>0.12070528049761524</v>
+      </c>
+      <c r="J305" s="2">
+        <v>81787.945000000007</v>
+      </c>
+      <c r="K305" s="2">
+        <v>53245.936000000002</v>
+      </c>
+      <c r="L305" s="2">
+        <v>50658.256000000001</v>
+      </c>
+      <c r="M305" s="2">
+        <v>2587.6799999999998</v>
+      </c>
+      <c r="N305" s="2">
+        <f t="shared" si="34"/>
+        <v>28542.009000000005</v>
+      </c>
+      <c r="O305" s="2">
+        <v>6114.7190000000001</v>
+      </c>
+      <c r="P305" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="306" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
         <v>847</v>
       </c>
@@ -17241,7 +17281,7 @@
       <c r="E306" s="48"/>
       <c r="O306" s="2"/>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
         <v>848</v>
       </c>
@@ -17256,7 +17296,7 @@
       </c>
       <c r="O307" s="2"/>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
         <v>849</v>
       </c>
@@ -17271,7 +17311,7 @@
       </c>
       <c r="O308" s="2"/>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
         <v>850</v>
       </c>
@@ -17286,7 +17326,7 @@
       </c>
       <c r="O309" s="2"/>
     </row>
-    <row r="310" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
         <v>851</v>
       </c>
@@ -17301,7 +17341,7 @@
       </c>
       <c r="O310" s="2"/>
     </row>
-    <row r="311" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
         <v>852</v>
       </c>
@@ -17316,7 +17356,7 @@
       </c>
       <c r="O311" s="2"/>
     </row>
-    <row r="312" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
         <v>853</v>
       </c>
@@ -50715,6 +50755,9 @@
       <c r="A197" s="1" t="s">
         <v>846</v>
       </c>
+      <c r="B197" t="s">
+        <v>864</v>
+      </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">

</xml_diff>